<commit_message>
UAT Term Life: reclassify API-validation cases as by-design; keep defects for plans/premium/covers/outputs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QHwJi3zeYQjFLvR25qEcTo
</commit_message>
<xml_diff>
--- a/UAT_TermLife/TermLife_UAT_TestCases_and_Results.xlsx
+++ b/UAT_TermLife/TermLife_UAT_TestCases_and_Results.xlsx
@@ -42,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -66,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -77,11 +77,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FF9999"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,6 +131,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -143,9 +141,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -516,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -562,7 +557,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>InsureMO back-end APIs (Postman collection) for product TL001 – Term Life with/without Travel. UI cases listed as Not Executed.</t>
+          <t>Plans, premium, covers and generated outputs (API has no input validation by design – validation cases are classed BY DESIGN). InsureMO back-end APIs (Postman collection) for product TL001 – Term Life with/without Travel. UI cases listed as Not Executed.</t>
         </is>
       </c>
     </row>
@@ -603,10 +598,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>24.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="9">
@@ -616,23 +611,23 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>14.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="11">
@@ -685,6 +680,11 @@
           <t>Observation</t>
         </is>
       </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>By design</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -704,6 +704,9 @@
       <c r="E15" t="n">
         <v>0</v>
       </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -718,10 +721,13 @@
         <v>12</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -737,11 +743,14 @@
         <v>27</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -756,11 +765,14 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
+      <c r="F18" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -778,7 +790,10 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -794,11 +809,14 @@
         <v>6</v>
       </c>
       <c r="D20" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
+      <c r="F20" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -813,11 +831,14 @@
         <v>11</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
       </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -832,11 +853,14 @@
         <v>5</v>
       </c>
       <c r="D22" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
+      <c r="F22" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -851,10 +875,13 @@
         <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="24">
@@ -870,11 +897,14 @@
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
+      <c r="F24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -894,6 +924,9 @@
       <c r="E25" t="n">
         <v>1</v>
       </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -913,6 +946,9 @@
       <c r="E26" t="n">
         <v>0</v>
       </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -930,6 +966,9 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -951,6 +990,9 @@
       <c r="E28" t="n">
         <v>0</v>
       </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -965,10 +1007,13 @@
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -984,10 +1029,13 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -1003,11 +1051,14 @@
         <v>6</v>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>3</v>
       </c>
+      <c r="F31" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1022,11 +1073,14 @@
         <v>8</v>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E32" t="n">
         <v>2</v>
       </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1046,6 +1100,9 @@
       <c r="E33" t="n">
         <v>1</v>
       </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1065,6 +1122,9 @@
       <c r="E34" t="n">
         <v>3</v>
       </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1079,9 +1139,12 @@
         <v>5</v>
       </c>
       <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>1</v>
       </c>
-      <c r="E35" t="n">
+      <c r="F35" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2090,12 +2153,12 @@
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Invalid ProductSubcode 3 → HTTP 200 with empty PlanList (no error returned). UI must handle empty plan list.</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Invalid ProductSubcode 3 → HTTP 200 with empty PlanList (no error returned). UI must handle empty plan list. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I22" s="8" t="n">
@@ -2135,12 +2198,12 @@
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Accepted without ChannelCode</t>
+          <t>[Was: FAIL] Accepted without ChannelCode | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I23" s="8" t="n">
@@ -2180,12 +2243,12 @@
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Accepted with unknown ChannelCode</t>
+          <t>[Was: FAIL] Accepted with unknown ChannelCode | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I24" s="8" t="n">
@@ -2228,7 +2291,7 @@
           <t>Plan 1 benefits total 31000 (DTH+PTD+PPD+REX) but policy/lob/risk SumInsured=62000; PlanList has 2 entries (2nd entry has no PlanId/PlanName – duplicate)</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -2495,12 +2558,12 @@
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Monthly mode (3) accepted for Term Life: PTL0010000000050 premium 216. Spec: Term Life = Annual and Single only (Monthly only for Life Protect).</t>
+          <t>[Was: FAIL] Monthly mode (3) accepted for Term Life: PTL0010000000050 premium 216. Spec: Term Life = Annual and Single only (Monthly only for Life Protect). | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I31" s="8" t="n">
@@ -3575,12 +3638,12 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>Annual mode with PolicyTerm=2 accepted (PTL0010000000051); spec: Annual = 1 year only</t>
+          <t>[Was: FAIL] Annual mode with PolicyTerm=2 accepted (PTL0010000000051); spec: Annual = 1 year only | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I55" s="8" t="n">
@@ -3620,12 +3683,12 @@
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>Single, term 2: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2028-10-12); PolicyTerm=2</t>
+          <t>[Was: FAIL] Single, term 2: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2028-10-12); PolicyTerm=2 | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I56" s="8" t="n">
@@ -3665,12 +3728,12 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>Single, term 5: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2031-10-12); PolicyTerm=5</t>
+          <t>[Was: FAIL] Single, term 5: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2031-10-12); PolicyTerm=5 | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I57" s="8" t="n">
@@ -3710,12 +3773,12 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>Single, term 10: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2036-10-12); PolicyTerm=10</t>
+          <t>[Was: FAIL] Single, term 10: premium 216, ExpiryDate 2027-10-12T23:59:59 (expected cover end 2036-10-12); PolicyTerm=10 | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I58" s="8" t="n">
@@ -3755,12 +3818,12 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>Single premium with term 0 accepted (PTL0010000000055); spec: Single term 2–10 (min/max configurable)</t>
+          <t>[Was: FAIL] Single premium with term 0 accepted (PTL0010000000055); spec: Single term 2–10 (min/max configurable) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I59" s="8" t="n">
@@ -3800,12 +3863,12 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>Single premium with term 11 accepted (PTL0010000000056); spec: Single term 2–10 (min/max configurable)</t>
+          <t>[Was: FAIL] Single premium with term 11 accepted (PTL0010000000056); spec: Single term 2–10 (min/max configurable) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I60" s="8" t="n">
@@ -3935,12 +3998,12 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>Backend accepted DOB 2008-10-14 (17y 364d – below min age 18). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth.</t>
-        </is>
-      </c>
-      <c r="H63" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Backend accepted DOB 2008-10-14 (17y 364d – below min age 18). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H63" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I63" s="8" t="n">
@@ -4070,12 +4133,12 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>Backend accepted DOB 1961-10-13 (exactly 65 – above max entry age 64). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth.</t>
-        </is>
-      </c>
-      <c r="H66" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Backend accepted DOB 1961-10-13 (exactly 65 – above max entry age 64). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I66" s="8" t="n">
@@ -4115,12 +4178,12 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>Backend accepted DOB 1957-10-14 (68y – above max entry 64). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth.</t>
-        </is>
-      </c>
-      <c r="H67" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Backend accepted DOB 1957-10-14 (68y – above max entry 64). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H67" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I67" s="8" t="n">
@@ -4160,12 +4223,12 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>Backend accepted DOB 1956-10-12 (70y – above max age 69 / exit 70). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth.</t>
-        </is>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Backend accepted DOB 1956-10-12 (70y – above max age 69 / exit 70). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H68" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I68" s="8" t="n">
@@ -4205,12 +4268,12 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>Backend accepted DOB 2030-01-01 (future date of birth). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth.</t>
-        </is>
-      </c>
-      <c r="H69" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Backend accepted DOB 2030-01-01 (future date of birth). Spec: age rules (min 18, max entry 64, max age 69, exit 70) are enforced by Uponly UI; backend enforcement absent – recommend defence-in-depth. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H69" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I69" s="8" t="n">
@@ -4295,12 +4358,12 @@
       </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000069 (mandatory field InsuredName omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000069 (mandatory field InsuredName omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H71" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I71" s="8" t="n">
@@ -4340,12 +4403,12 @@
       </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000070 (mandatory field DateOfBirth omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000070 (mandatory field DateOfBirth omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I72" s="8" t="n">
@@ -4385,12 +4448,12 @@
       </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000071 (mandatory field Gender omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000071 (mandatory field Gender omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H73" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I73" s="8" t="n">
@@ -4430,12 +4493,12 @@
       </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000072 (mandatory field IdNo omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000072 (mandatory field IdNo omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H74" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I74" s="8" t="n">
@@ -4475,12 +4538,12 @@
       </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000073 (mandatory field IdType omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000073 (mandatory field IdType omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H75" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I75" s="8" t="n">
@@ -4520,12 +4583,12 @@
       </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000074 (mandatory field Salutation omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000074 (mandatory field Salutation omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I76" s="8" t="n">
@@ -4565,12 +4628,12 @@
       </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000075 (mandatory field ResidentStatus omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000075 (mandatory field ResidentStatus omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H77" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I77" s="8" t="n">
@@ -4610,12 +4673,12 @@
       </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000076 (mandatory field Email omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000076 (mandatory field Email omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I78" s="8" t="n">
@@ -4655,12 +4718,12 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000077 (mandatory field Mobile omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000077 (mandatory field Mobile omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H79" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I79" s="8" t="n">
@@ -4700,12 +4763,12 @@
       </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000078 (mandatory field MaritalStatus omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000078 (mandatory field MaritalStatus omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H80" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I80" s="8" t="n">
@@ -4745,12 +4808,12 @@
       </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000079 (mandatory field Address omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000079 (mandatory field Address omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H81" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I81" s="8" t="n">
@@ -4790,12 +4853,12 @@
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000080 (CIFNumber omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000080 (CIFNumber omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I82" s="8" t="n">
@@ -4835,12 +4898,12 @@
       </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000081 (CustomerType omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000081 (CustomerType omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H83" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I83" s="8" t="n">
@@ -4880,12 +4943,12 @@
       </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000082 (BranchCode omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000082 (BranchCode omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I84" s="8" t="n">
@@ -4970,12 +5033,12 @@
       </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000083 (PremiumModeCode omitted)</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000083 (PremiumModeCode omitted) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I86" s="8" t="n">
@@ -5195,12 +5258,12 @@
       </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000095 invalid email</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000095 invalid email | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H91" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I91" s="8" t="n">
@@ -5240,12 +5303,12 @@
       </c>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000096 alphabetic mobile</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000096 alphabetic mobile | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H92" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I92" s="8" t="n">
@@ -5285,12 +5348,12 @@
       </c>
       <c r="G93" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000097 negative salary</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000097 negative salary | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H93" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I93" s="8" t="n">
@@ -5375,12 +5438,12 @@
       </c>
       <c r="G95" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000099 300-char name</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000099 300-char name | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H95" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I95" s="8" t="n">
@@ -5555,12 +5618,12 @@
       </c>
       <c r="G99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000089 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000089  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H99" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I99" s="8" t="n">
@@ -5870,12 +5933,12 @@
       </c>
       <c r="G106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000094 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000094  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I106" s="8" t="n">
@@ -6095,12 +6158,12 @@
       </c>
       <c r="G111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000107 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000107  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H111" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I111" s="8" t="n">
@@ -6140,12 +6203,12 @@
       </c>
       <c r="G112" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000108 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000108  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H112" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I112" s="8" t="n">
@@ -6185,12 +6248,12 @@
       </c>
       <c r="G113" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000109 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000109  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H113" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I113" s="8" t="n">
@@ -6230,12 +6293,12 @@
       </c>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000110 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000110  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H114" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I114" s="8" t="n">
@@ -6275,12 +6338,12 @@
       </c>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000111 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000111  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H115" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I115" s="8" t="n">
@@ -6410,12 +6473,12 @@
       </c>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Accepted (HTTP 200) and created PTL0010000000113 </t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000113  | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H118" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I118" s="8" t="n">
@@ -6545,12 +6608,12 @@
       </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t>Policy POTL00100000003 issued without LC Code / LG Code / Debit details (spec: mandatory before policy conversion)</t>
+          <t>[Was: FAIL] Policy POTL00100000003 issued without LC Code / LG Code / Debit details (spec: mandatory before policy conversion) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H121" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I121" s="8" t="n">
@@ -6635,12 +6698,12 @@
       </c>
       <c r="G123" s="8" t="inlineStr">
         <is>
-          <t>LGCode 'ZZ' (arbitrary) accepted – LG/LC codes are not validated against a master list.</t>
-        </is>
-      </c>
-      <c r="H123" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] LGCode 'ZZ' (arbitrary) accepted – LG/LC codes are not validated against a master list. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H123" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I123" s="8" t="n">
@@ -6680,12 +6743,12 @@
       </c>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000101 expiry before effective</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000101 expiry before effective | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H124" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I124" s="8" t="n">
@@ -6725,12 +6788,12 @@
       </c>
       <c r="G125" s="8" t="inlineStr">
         <is>
-          <t>Accepted (HTTP 200) and created PTL0010000000102 back-dated effective date</t>
+          <t>[Was: FAIL] Accepted (HTTP 200) and created PTL0010000000102 back-dated effective date | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H125" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I125" s="8" t="n">
@@ -7355,12 +7418,12 @@
       </c>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t>Non-existent ProposalNo → HTTP 200 with body validateResult.errors[]: 'Proposal not found for proposal no: …'. Error is carried in a 200 body (other APIs use 400/404) – consumers must inspect body.</t>
-        </is>
-      </c>
-      <c r="H139" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Non-existent ProposalNo → HTTP 200 with body validateResult.errors[]: 'Proposal not found for proposal no: …'. Error is carried in a 200 body (other APIs use 400/404) – consumers must inspect body. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H139" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I139" s="8" t="n">
@@ -7400,12 +7463,12 @@
       </c>
       <c r="G140" s="8" t="inlineStr">
         <is>
-          <t>Missing identifiers → HTTP 200 with body validateResult.errors[]: 'quotationNo, proposalNo, or policyNo parameter is missing.' (HTTP 200 for an error).</t>
-        </is>
-      </c>
-      <c r="H140" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Missing identifiers → HTTP 200 with body validateResult.errors[]: 'quotationNo, proposalNo, or policyNo parameter is missing.' (HTTP 200 for an error). | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H140" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I140" s="8" t="n">
@@ -7805,12 +7868,12 @@
       </c>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t>Non-existent PolicyNo → HTTP 500 and raw Java NPE text leaked: 'Cannot invoke "java.util.Map.get(Object)" because "policyResponse" is null'. Should be a clean 404.</t>
-        </is>
-      </c>
-      <c r="H149" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Non-existent PolicyNo → HTTP 500 and raw Java NPE text leaked: 'Cannot invoke "java.util.Map.get(Object)" because "policyResponse" is null'. Should be a clean 404. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H149" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I149" s="8" t="n">
@@ -7850,12 +7913,12 @@
       </c>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t>Policy readable via a different ChannelCode (data isolation)</t>
+          <t>[Was: FAIL] Policy readable via a different ChannelCode (data isolation) | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H150" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I150" s="8" t="n">
@@ -7940,12 +8003,12 @@
       </c>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t>CONFIRMED on re-test: proposal rejected (reject API → SUCCESS, ProposalStatus=4) and then issue API → HTTP 200, PolicyNo POTL00100000016 generated, PolicyStatus=2 (Effective), ProposalStatus=3. A rejected proposal must not be issuable.</t>
+          <t>[Was: FAIL] CONFIRMED on re-test: proposal rejected (reject API → SUCCESS, ProposalStatus=4) and then issue API → HTTP 200, PolicyNo POTL00100000016 generated, PolicyStatus=2 (Effective), ProposalStatus=3. A rejected proposal must not be issuable. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I152" s="8" t="n">
@@ -8075,12 +8138,12 @@
       </c>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t>Reject without ProposalRejectDesc → HTTP 200 'Proposal rejected' (status 4). Spec: 'Enter comments if any' (optional) – accepted as designed; recommend mandatory reason for audit.</t>
-        </is>
-      </c>
-      <c r="H155" s="10" t="inlineStr">
-        <is>
-          <t>OBSERVATION</t>
+          <t>[Was: OBSERVATION] Reject without ProposalRejectDesc → HTTP 200 'Proposal rejected' (status 4). Spec: 'Enter comments if any' (optional) – accepted as designed; recommend mandatory reason for audit. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
+        </is>
+      </c>
+      <c r="H155" s="11" t="inlineStr">
+        <is>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I155" s="8" t="n">
@@ -8348,7 +8411,7 @@
           <t>English cancellation clause renders '8096 of the unearned Premium' (should read 80%); Arabic side shows 80%. Page footer 'Page 2 of 3' also truncated.</t>
         </is>
       </c>
-      <c r="H161" s="11" t="inlineStr">
+      <c r="H161" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -8525,12 +8588,12 @@
       </c>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t>Certificate request for non-existent PolicyNo POTL00199999999 → HTTP 200 and a BLANK certificate PDF (all fields empty) instead of an error.</t>
+          <t>[Was: FAIL] Certificate request for non-existent PolicyNo POTL00199999999 → HTTP 200 and a BLANK certificate PDF (all fields empty) instead of an error. | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H165" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I165" s="8" t="n">
@@ -8570,12 +8633,12 @@
       </c>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t>Certificate request using an un-issued ProposalNo → HTTP 200 and a BLANK certificate PDF instead of an error (certificate should exist only after issue).</t>
+          <t>[Was: FAIL] Certificate request using an un-issued ProposalNo → HTTP 200 and a BLANK certificate PDF instead of an error (certificate should exist only after issue). | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H166" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I166" s="8" t="n">
@@ -8753,7 +8816,7 @@
           <t>Missing from feed vs spec 'Feed File' sheet: ['Branch Code', 'LCCode', 'LGCode']</t>
         </is>
       </c>
-      <c r="H170" s="11" t="inlineStr">
+      <c r="H170" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -8798,7 +8861,7 @@
           <t>Product Name values for TL001 policies: ['Personal Accident with TTD', 'Personal Accident without TTD']</t>
         </is>
       </c>
-      <c r="H171" s="11" t="inlineStr">
+      <c r="H171" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -8843,7 +8906,7 @@
           <t>6 of 6 Effective (non-cancelled) policies have a Cancelled Date populated, e.g. ['POTL00100000007', 'POTL00100000006', 'POTL00100000005']</t>
         </is>
       </c>
-      <c r="H172" s="11" t="inlineStr">
+      <c r="H172" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -9200,12 +9263,12 @@
       </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t>xlsx returned for invalid module</t>
+          <t>[Was: FAIL] xlsx returned for invalid module | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H180" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I180" s="8" t="n">
@@ -9428,7 +9491,7 @@
           <t>Free-look configured as 15 days (cancel-check PremiumDetails.FreeLookDays=15). Application form states a 30-day Review Period with full refund.</t>
         </is>
       </c>
-      <c r="H185" s="11" t="inlineStr">
+      <c r="H185" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10193,7 +10256,7 @@
           <t>cancel-check / cancel-approve responses return CarrierName 'Afillar Insurance Company' (code AFIC) whereas application form and certificate show 'Arabia Falcon Insurance SAOG'.</t>
         </is>
       </c>
-      <c r="H202" s="11" t="inlineStr">
+      <c r="H202" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10238,7 +10301,7 @@
           <t>Policy with pending request POTL00100000017-001 (created for 2026-10-13, FREE_LOOK refund 216): subsequent cancel-check calls for 2026-10-20, 2027-01-13 and again 2026-10-13 all return the SAME stale data (day 0, FREE_LOOK, 216). Date validation (before commencement / after expiry) is also bypassed once a request is pending (observed accepted in main run).</t>
         </is>
       </c>
-      <c r="H203" s="11" t="inlineStr">
+      <c r="H203" s="12" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
@@ -10685,12 +10748,12 @@
       </c>
       <c r="G213" s="8" t="inlineStr">
         <is>
-          <t>Validation failures return HTTP [500, 200, 200] — all business-validation errors surface as HTTP 500 INTERNAL_ERROR instead of 4xx with field-level messages</t>
+          <t>[Was: FAIL] Validation failures return HTTP [500, 200, 200] — all business-validation errors surface as HTTP 500 INTERNAL_ERROR instead of 4xx with field-level messages | By design – the API performs no input validation; Uponly UI must enforce. Recorded as a risk, not a defect.</t>
         </is>
       </c>
       <c r="H213" s="11" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>BY DESIGN</t>
         </is>
       </c>
       <c r="I213" s="8" t="n">
@@ -10778,7 +10841,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H215" s="12" t="inlineStr">
+      <c r="H215" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -10821,7 +10884,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H216" s="12" t="inlineStr">
+      <c r="H216" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -10864,7 +10927,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI + CIF API)</t>
         </is>
       </c>
-      <c r="H217" s="12" t="inlineStr">
+      <c r="H217" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -10907,7 +10970,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H218" s="12" t="inlineStr">
+      <c r="H218" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -10950,7 +11013,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H219" s="12" t="inlineStr">
+      <c r="H219" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -10993,7 +11056,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H220" s="12" t="inlineStr">
+      <c r="H220" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11036,7 +11099,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H221" s="12" t="inlineStr">
+      <c r="H221" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11079,7 +11142,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H222" s="12" t="inlineStr">
+      <c r="H222" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11122,7 +11185,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H223" s="12" t="inlineStr">
+      <c r="H223" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11165,7 +11228,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H224" s="12" t="inlineStr">
+      <c r="H224" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11208,7 +11271,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H225" s="12" t="inlineStr">
+      <c r="H225" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11251,7 +11314,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H226" s="12" t="inlineStr">
+      <c r="H226" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11294,7 +11357,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H227" s="12" t="inlineStr">
+      <c r="H227" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11337,7 +11400,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H228" s="12" t="inlineStr">
+      <c r="H228" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11380,7 +11443,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H229" s="12" t="inlineStr">
+      <c r="H229" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11423,7 +11486,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H230" s="12" t="inlineStr">
+      <c r="H230" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11466,7 +11529,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H231" s="12" t="inlineStr">
+      <c r="H231" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11509,7 +11572,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H232" s="12" t="inlineStr">
+      <c r="H232" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11552,7 +11615,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H233" s="12" t="inlineStr">
+      <c r="H233" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11595,7 +11658,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H234" s="12" t="inlineStr">
+      <c r="H234" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11638,7 +11701,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H235" s="12" t="inlineStr">
+      <c r="H235" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11681,7 +11744,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H236" s="12" t="inlineStr">
+      <c r="H236" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11724,7 +11787,7 @@
           <t>Not executed – requires Uponly UI (Uponly UI)</t>
         </is>
       </c>
-      <c r="H237" s="12" t="inlineStr">
+      <c r="H237" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11767,7 +11830,7 @@
           <t>Not executed – requires Uponly UI (Business TBD)</t>
         </is>
       </c>
-      <c r="H238" s="12" t="inlineStr">
+      <c r="H238" s="13" t="inlineStr">
         <is>
           <t>NOT EXECUTED</t>
         </is>
@@ -11786,7 +11849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -11847,39 +11910,39 @@
           <t>DEF-01</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Proposal Reject / Issue</t>
+          <t>Create Proposal</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>A rejected proposal can still be issued as an Effective policy</t>
+          <t>Sum Insured is double-counted – PlanList contains a duplicate, empty plan entry</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Create proposal → proposal-reject (SUCCESS, ProposalStatus=4) → issue returns HTTP 200 with a new PolicyNo (POTL00100000016, PolicyStatus=2). Checker rejection is bypassable; business control failure.</t>
+          <t>Every proposal response contains 2 PlanList entries (2nd has no PlanId/PlanName but all coverages). Policy/LOB/Risk SumInsured = 2× the selected plan (Plan 1 With Travel: 62,000 instead of 31,000; Plan 2: 122,000 instead of 61,000).</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Policy Lifecycle – Approval Process (approve or reject)</t>
+          <t>Coverages and Sum Assured sheet</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>TL-REJ-02</t>
+          <t>TL-PREM-90</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Block issue (and update) when ProposalStatus = Rejected; return a clear 4xx.</t>
+          <t>Return only the selected plan; fix SumInsured roll-up. Verify Production Report / feed totals are not affected.</t>
         </is>
       </c>
     </row>
@@ -11889,39 +11952,39 @@
           <t>DEF-02</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Issue / Payment</t>
+          <t>Feed File</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Policy can be issued without LC Code, LG Code or payment/debit details</t>
+          <t>Product Name in feed is wrong for Term Life policies</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Proposal saved without PolicyPaymentInfoList and then issued → POTL00100000003 Effective. Spec: LC Code, LG Code, Premium mandatory before policy conversion.</t>
+          <t>Feed rows for TL001 policies show 'Personal Accident with TTD' / 'Personal Accident without TTD'. Expected 'Term Life with Travel' / 'Term Life without Travel'.</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Fields sheet – LC Code / LG Code 'Mandatory (before policy conversion)'</t>
+          <t>Feed File sheet – Product Name</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>TL-PAY-01, TL-PAY-02, TL-PAY-04</t>
+          <t>TL-FEED-03</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Enforce mandatory payment fields (and validate LG/LC against master) in the issue step.</t>
+          <t>Fix product-name mapping (ProductSubcode → name) in feed template.</t>
         </is>
       </c>
     </row>
@@ -11931,39 +11994,39 @@
           <t>DEF-03</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Create Proposal</t>
+          <t>Feed File</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Sum Insured is double-counted – PlanList contains a duplicate, empty plan entry</t>
+          <t>Cancelled Date populated for non-cancelled (Effective) policies</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Every proposal response contains 2 PlanList entries (2nd has no PlanId/PlanName but all coverages). Policy/LOB/Risk SumInsured = 2× the selected plan (Plan 1 With Travel: 62,000 instead of 31,000; Plan 2: 122,000 instead of 61,000).</t>
+          <t>6 of 6 Effective policies in the feed carry a Cancelled Date equal to the issue timestamp.</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Coverages and Sum Assured sheet</t>
+          <t>Feed File sheet – Cancelled Date</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>TL-PREM-90</t>
+          <t>TL-FEED-04</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Return only the selected plan; fix SumInsured roll-up. Verify Production Report / feed totals are not affected.</t>
+          <t>Populate only when policy status = Cancelled.</t>
         </is>
       </c>
     </row>
@@ -11973,39 +12036,39 @@
           <t>DEF-04</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Feed File</t>
+          <t>Cancellation</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Product Name in feed is wrong for Term Life policies</t>
+          <t>Repeat cancel-check on a pending request returns stale refund data for the old date</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Feed rows for TL001 policies show 'Personal Accident with TTD' / 'Personal Accident without TTD'. Expected 'Term Life with Travel' / 'Term Life without Travel'.</t>
+          <t>After the first cancel-check creates a PENDING request, later calls with a different CancellationDate return the first request's calculation (e.g. day 0 / FREE_LOOK 216 even for 2027-01-13), so the refund shown is for the wrong date.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Feed File sheet – Product Name</t>
+          <t>Policy Lifecycle / cancellation flow</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>TL-FEED-03</t>
+          <t>TL-CAN-21</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Fix product-name mapping (ProductSubcode → name) in feed template.</t>
+          <t>Recalculate and validate each request, or reject with 'request already pending'.</t>
         </is>
       </c>
     </row>
@@ -12015,39 +12078,39 @@
           <t>DEF-05</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Feed File</t>
+          <t>Cancellation / Documents</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Cancelled Date populated for non-cancelled (Effective) policies</t>
+          <t>Free-look period mismatch: system 15 days vs application form 30 days</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>6 of 6 Effective policies in the feed carry a Cancelled Date equal to the issue timestamp.</t>
+          <t>cancel-check FreeLookDays=15; Day-15 cancellation falls to pro-rata. Application form 'Review Period' promises full refund within 30 days.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Feed File sheet – Cancelled Date</t>
+          <t>Application form – Review Period</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>TL-FEED-04</t>
+          <t>TL-CAN-03</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Populate only when policy status = Cancelled.</t>
+          <t>Align configuration with the form (or correct the form).</t>
         </is>
       </c>
     </row>
@@ -12057,39 +12120,39 @@
           <t>DEF-06</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Beneficiary</t>
+          <t>Cancellation</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Beneficiary share total is not validated</t>
+          <t>Carrier name inconsistent: 'Afillar Insurance Company' vs 'Arabia Falcon Insurance'</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Shares 50 (single), 60+60, 150, -100 and a blank beneficiary name were all accepted. Forms state 'Share % (total to equal 100%)'.</t>
+          <t>cancel-check and cancel-approve return CarrierCode AFIC / 'Afillar Insurance Company'; certificate and application form show 'Arabia Falcon Insurance SAOG'.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Application form / Fields – Beneficiary</t>
+          <t>Certificate / Application format</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>TL-BEN-03..07, TL-BEN-10</t>
+          <t>TL-CAN-20</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Validate Σshare = 100, each 0&lt;share≤100, name mandatory, at least one beneficiary.</t>
+          <t>Correct carrier master data / notification templates.</t>
         </is>
       </c>
     </row>
@@ -12099,39 +12162,39 @@
           <t>DEF-07</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Field Validation</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Mandatory fields are not enforced by the back-end</t>
+          <t>Application form: English cancellation clause prints '8096 of the unearned Premium'; footer 'Page 2 of 3' truncated</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Proposal created successfully with InsuredName, DateOfBirth, Gender, IdNo, IdType, Salutation, ResidentStatus, Email, Mobile, MaritalStatus, Address, CIFNumber, CustomerType, BranchCode or PremiumModeCode omitted (14 of 16 tested). Only PlanId is enforced (via an iHub exception).</t>
+          <t>Static clause renders '80%' as '8096' on page 2 of the generated application form (Arabic side correct). Page-number footer is clipped.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Fields sheet – 'Mandatory' flags</t>
+          <t>Application form format</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>TL-VAL-01..14, TL-VAL-16</t>
+          <t>TL-DOC-05</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Add mandatory-field validation in the Create/Update Proposal API (UI-only validation is bypassable).</t>
+          <t>Fix the template (escape '%' / font) and footer width.</t>
         </is>
       </c>
     </row>
@@ -12141,457 +12204,37 @@
           <t>DEF-08</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Premium Mode</t>
+          <t>Feed File</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Monthly premium mode accepted for Term Life</t>
+          <t>Feed file is missing Branch Code, LCCode and LGCode columns</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>PremiumModeCode=3 creates a TL proposal (premium unchanged at 216). Monthly is meant only for Life Protect; Term Life = Annual &amp; Single.</t>
+          <t>Feed has 27 columns; spec lists 30 (Branch Code, LCCode, LGCode absent).</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Premium &amp; Rates / LOV – Premium Mode is product-wise</t>
+          <t>Feed File sheet</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>TL-PREM-96</t>
+          <t>TL-FEED-02</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Restrict PremiumMode by product (configurable).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>DEF-09</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Policy term / expiry not validated or derived</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Annual with term 2, Single with term 0 and 11 accepted; PolicyTerm and ExpiryDate are independent (term 5 with 1-year expiry accepted). With a consistent expiry the certificate is correct (TL-TERM-08).</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Fields sheet – Term (Single 2–10 yrs; min/max configurable per product)</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>TL-TERM-01..06</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Derive ExpiryDate from term; enforce Annual=1 and Single min/max (configurable).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>DEF-10</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Field Validation</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Data-quality validations missing</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Accepted: invalid email, alphabetic mobile, negative salary, 300-char name, IdType=9, MaritalStatus=9, ExpiryDate earlier than EffectiveDate, back-dated EffectiveDate.</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Fields sheet / LOV fields</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>TL-VAL-30,31,32,34, TL-LOV-24, TL-LOV-31, TL-DATE-01, TL-DATE-02</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Add format/range/code-table validation; reject illogical dates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>DEF-11</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Cancellation</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Repeat cancel-check on a pending request returns stale data and skips validation</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>After the first cancel-check creates a PENDING request, later calls with different CancellationDate return the first request's calculation (e.g. day 0 / FREE_LOOK 216 even for a 2027-01-13 date) and bypass before-commencement / after-expiry checks.</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Policy Lifecycle / cancellation flow</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>TL-CAN-21 (masked TL-CAN-05/06 in first run)</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Recalculate and validate each request, or reject with 'request already pending'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>DEF-12</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Cancellation / Documents</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Free-look period mismatch: system 15 days vs application form 30 days</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>cancel-check FreeLookDays=15; Day-15 cancellation falls to pro-rata. Application form 'Review Period' promises full refund within 30 days.</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Application form – Review Period</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>TL-CAN-03</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Align configuration with the form (or correct the form).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>DEF-13</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Cancellation</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Carrier name inconsistent: 'Afillar Insurance Company' vs 'Arabia Falcon Insurance'</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>cancel-check and cancel-approve return CarrierCode AFIC / 'Afillar Insurance Company'; certificate and application form show 'Arabia Falcon Insurance SAOG'.</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Certificate / Application format</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>TL-CAN-20</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Correct carrier master data / notification templates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>DEF-14</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Documents</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Application form: English cancellation clause prints '8096 of the unearned Premium'; footer 'Page 2 of 3' truncated</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Static clause renders '80%' as '8096' on page 2 of the generated application form (Arabic side correct). Page-number footer is clipped.</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Application form format</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>TL-DOC-05</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Fix the template (escape '%' / font) and footer width.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>DEF-15</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Documents</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Blank certificate generated for non-existent policy and for un-issued proposal</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>doc_generation DocType=Policy returns HTTP 200 + empty-field PDF for POTL00199999999 and for a PTL… proposal number.</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Policy Lifecycle – certificate printed after approval</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>TL-DOC-09, TL-DOC-10</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Return 404/400 when policy not found or not issued.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>DEF-16</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>API Error Handling</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Business-validation errors return HTTP 500 INTERNAL_ERROR and leak internal details</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Invalid codes/plan/product etc. return HTTP 500 with iHub URLs, Java exceptions (e.g. NPE text in load-policy for unknown policy). Some not-found cases return HTTP 200 with validateResult.errors. Cancellation APIs, by contrast, return proper 400/404/409.</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>TL-NFR-06, TL-POL-02, TL-LOAD-02/03, TL-PLAN-12</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Standardise to 4xx with field-level messages; hide internal stack/URLs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>DEF-17</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Security</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>ChannelCode not enforced as a data boundary</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
-        <is>
-          <t>get-plans accepts a missing or unknown ChannelCode; an issued policy can be loaded with ChannelCode=OTHER.</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>General – channel-based access</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>TL-PLAN-14, TL-PLAN-15, TL-POL-03</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Validate ChannelCode against the token's channel and scope data access.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>DEF-18</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Feed File</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Feed missing Branch Code, LCCode, LGCode columns; invalid Module accepted</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>Feed has 27 columns; spec lists 30. Module='Nope' still returns an xlsx.</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Feed File sheet</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>TL-FEED-02, TL-FEED-12</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>Add the three columns; validate Module.</t>
         </is>

</xml_diff>